<commit_message>
Before sigmoid actuation function 1/15/2026
</commit_message>
<xml_diff>
--- a/Preliminary Data/two forces (SVD optimized)/Validation(SVD)(3tendon).xlsx
+++ b/Preliminary Data/two forces (SVD optimized)/Validation(SVD)(3tendon).xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://djpropertycom-my.sharepoint.com/personal/noah_familiajones_org/Documents/Work and Projects/Github/Whisker_Inspired_Sensing_CR/Raw Data/two forces (SVD optimized)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://djpropertycom-my.sharepoint.com/personal/noah_familiajones_org/Documents/Work and Projects/Github/Whisker_Inspired_Sensing_CR/Preliminary Data/two forces (SVD optimized)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3483" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7D1A446-FD79-4D87-9F59-3F514B506D32}"/>
+  <xr:revisionPtr revIDLastSave="3489" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A344F4BF-760C-43C9-A634-5FA9BB325913}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3D16C37F-3C74-4527-A308-796C339DFE9F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3D16C37F-3C74-4527-A308-796C339DFE9F}"/>
   </bookViews>
   <sheets>
     <sheet name="Proximal Validation (empirical)" sheetId="12" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -893,7 +893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B763EDC-8536-442D-A8D3-F37978D4DE80}">
-  <dimension ref="A1:AB22"/>
+  <dimension ref="A1:AB33"/>
   <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
@@ -2316,50 +2316,136 @@
         <v>9.1469999999999996E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20">
-        <v>0.78500000000000003</v>
-      </c>
-      <c r="D20">
-        <v>45</v>
-      </c>
-      <c r="F20">
-        <v>1.0469999999999999</v>
-      </c>
-      <c r="G20">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21">
-        <v>2.6179999999999999</v>
-      </c>
-      <c r="D21">
-        <v>150</v>
-      </c>
-      <c r="F21">
-        <v>2.3559999999999999</v>
-      </c>
-      <c r="G21">
-        <v>135</v>
-      </c>
-    </row>
     <row r="22" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22">
-        <v>3.927</v>
-      </c>
-      <c r="D22">
-        <v>225</v>
-      </c>
-      <c r="F22">
-        <v>3.665</v>
-      </c>
-      <c r="G22">
-        <v>210</v>
-      </c>
       <c r="V22">
         <f>_xlfn.STDEV.S(V3,V7,V8,V9,V10)</f>
         <v>3.0729533123933337E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V26">
+        <v>5.5469816942511152E-3</v>
+      </c>
+      <c r="W26">
+        <v>7.4890812985151933E-3</v>
+      </c>
+      <c r="X26">
+        <v>-1.7669518729107575E-2</v>
+      </c>
+      <c r="Y26">
+        <v>-9.0311743283908175E-2</v>
+      </c>
+      <c r="Z26">
+        <v>-4.9859250386685705E-3</v>
+      </c>
+      <c r="AA26">
+        <v>3.1337790008225341E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V27">
+        <v>-2.4984329231497356E-3</v>
+      </c>
+      <c r="W27">
+        <v>6.8043089930117095E-4</v>
+      </c>
+      <c r="X27">
+        <v>9.2293666881208408E-3</v>
+      </c>
+      <c r="Y27">
+        <v>-8.1619476339206354E-2</v>
+      </c>
+      <c r="Z27">
+        <v>8.2082095580302827E-3</v>
+      </c>
+      <c r="AA27">
+        <v>-2.4618569075221808E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V28">
+        <v>2.9512642192965803E-3</v>
+      </c>
+      <c r="W28">
+        <v>-7.723656751856961E-3</v>
+      </c>
+      <c r="X28">
+        <v>9.5036795044503575E-3</v>
+      </c>
+      <c r="Y28">
+        <v>8.1952452070606252E-2</v>
+      </c>
+      <c r="Z28">
+        <v>7.4491156908347289E-2</v>
+      </c>
+      <c r="AA28">
+        <v>5.3675567093620091E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V29">
+        <v>-2.3432304519013309E-4</v>
+      </c>
+      <c r="W29">
+        <v>1.3278805888743282E-2</v>
+      </c>
+      <c r="X29">
+        <v>-1.0943418877370839E-2</v>
+      </c>
+      <c r="Y29">
+        <v>3.5997785836162921E-3</v>
+      </c>
+      <c r="Z29">
+        <v>-4.4505966608498426E-2</v>
+      </c>
+      <c r="AA29">
+        <v>-4.56485552646477E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V30">
+        <v>8.2255703700906055E-4</v>
+      </c>
+      <c r="W30">
+        <v>1.0653034889324849E-2</v>
+      </c>
+      <c r="X30">
+        <v>-1.4234149511327746E-2</v>
+      </c>
+      <c r="Y30">
+        <v>-7.8725195334451339E-2</v>
+      </c>
+      <c r="Z30">
+        <v>-3.0921821417347589E-2</v>
+      </c>
+      <c r="AA30">
+        <v>-3.0702713926019462E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="22:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V33">
+        <f>_xlfn.STDEV.S(V26:V30)</f>
+        <v>3.0729533123933337E-3</v>
+      </c>
+      <c r="W33">
+        <f t="shared" ref="W33:AA33" si="20">_xlfn.STDEV.S(W26:W30)</f>
+        <v>8.4729514053678758E-3</v>
+      </c>
+      <c r="X33">
+        <f t="shared" si="20"/>
+        <v>1.3169899969181951E-2</v>
+      </c>
+      <c r="Y33">
+        <f t="shared" si="20"/>
+        <v>7.4654019892859622E-2</v>
+      </c>
+      <c r="Z33">
+        <f t="shared" si="20"/>
+        <v>4.6306214138634248E-2</v>
+      </c>
+      <c r="AA33">
+        <f t="shared" si="20"/>
+        <v>4.3141403867623787E-2</v>
       </c>
     </row>
   </sheetData>
@@ -7590,23 +7676,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E12580AD17ADB64691A1BA4C2E042DA4" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6532fc6a52f3455fe895a4f720bca71c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xmlns:ns4="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9a2f75daf18a7097de825f86ff3fec6" ns3:_="" ns4:_="">
     <xsd:import namespace="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
@@ -7859,10 +7928,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D595912-0053-4104-933F-CDA3B3DBC546}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65923CC5-95C4-4597-AADE-A0DCE38786F0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
+    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7885,20 +7982,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65923CC5-95C4-4597-AADE-A0DCE38786F0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D595912-0053-4104-933F-CDA3B3DBC546}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
-    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>